<commit_message>
feat(stage2): automatic true/false grading (no manual facilitator step) (#2)
The 5+5+5 true/false-with-correction grading is now AUTOMATIC at submission, no
facilitator buttons needed:
- +5 marked-wrong: statement is false AND player chose خطأ (deterministic).
- +5 wrong-part: player's selected segment matches the question's expectedWrongPart
  (new optional 'targetPart' Excel column); if none given, accepts any real segment
  of the statement.
- +5 correction: player's correction matches expectedCorrection.
Comparison uses the shared Arabic normalizer (ignores diacritics/AL/separators).
Answers are saved gradingComplete=true, so the manual grading panel no longer
appears. Added expectedWrongPart to the type + parser; the 150-question Bible bank
now supplies the wrong part for its false statements (regenerated xlsx).

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/public/templates/sufaraa-bible-bank.xlsx
+++ b/public/templates/sufaraa-bible-bank.xlsx
@@ -6248,7 +6248,7 @@
         <v/>
       </c>
       <c r="S95" t="str">
-        <v/>
+        <v>موسى</v>
       </c>
       <c r="T95" t="str">
         <v/>
@@ -6372,7 +6372,7 @@
         <v/>
       </c>
       <c r="S97" t="str">
-        <v/>
+        <v>الناصرة</v>
       </c>
       <c r="T97" t="str">
         <v/>
@@ -6496,7 +6496,7 @@
         <v/>
       </c>
       <c r="S99" t="str">
-        <v/>
+        <v>بطرس</v>
       </c>
       <c r="T99" t="str">
         <v/>
@@ -6620,7 +6620,7 @@
         <v/>
       </c>
       <c r="S101" t="str">
-        <v/>
+        <v>إبراهيم</v>
       </c>
       <c r="T101" t="str">
         <v/>
@@ -6744,7 +6744,7 @@
         <v/>
       </c>
       <c r="S103" t="str">
-        <v/>
+        <v>الفلك</v>
       </c>
       <c r="T103" t="str">
         <v/>

</xml_diff>